<commit_message>
Recalibrate battery deployment parameter
</commit_message>
<xml_diff>
--- a/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
+++ b/InputData/elec/GBCGpUNR/Grid Bat Cap Growth per Unit Net Revenue.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\GBCGpUNR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8DA9D0-EE68-424C-8BE8-C34249865C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADBBF3F-9F82-4B8B-B5E5-882630F9B4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
+    <workbookView xWindow="4545" yWindow="3765" windowWidth="21600" windowHeight="12645" xr2:uid="{7E47E401-4FF2-4F75-986A-BA871D3584BD}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -427,14 +427,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1BF9ED0-8E48-4355-BDAD-C352BC3B92D2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -442,7 +442,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -458,12 +458,12 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="62.81640625" customWidth="1"/>
+    <col min="1" max="1" width="62.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -471,7 +471,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>

</xml_diff>